<commit_message>
Updates to output expedition files
</commit_message>
<xml_diff>
--- a/E6 Curacao.xlsx
+++ b/E6 Curacao.xlsx
@@ -12,7 +12,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="194" uniqueCount="114">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="201" uniqueCount="116">
   <si>
     <t>tissueID</t>
   </si>
@@ -245,6 +245,9 @@
     <t>basisOfRecord</t>
   </si>
   <si>
+    <t>sampleEnteredBy</t>
+  </si>
+  <si>
     <t>expedition</t>
   </si>
   <si>
@@ -317,7 +320,7 @@
     <t>Vega Thurber Lab</t>
   </si>
   <si>
-    <t xml:space="preserve"> OSU</t>
+    <t>OSU</t>
   </si>
   <si>
     <t>sed 1 (deep)</t>
@@ -351,6 +354,9 @@
   </si>
   <si>
     <t>EnvironmentalDNA</t>
+  </si>
+  <si>
+    <t>Colin Howe|Vivian Li|Eric Crandall</t>
   </si>
   <si>
     <t>E6</t>
@@ -637,25 +643,28 @@
       <c r="CA1" t="s">
         <v>77</v>
       </c>
+      <c r="CB1" t="s">
+        <v>78</v>
+      </c>
     </row>
     <row r="2">
       <c r="A2" t="s">
-        <v>78</v>
+        <v>79</v>
       </c>
       <c r="B2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="C2" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D2" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E2" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F2" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G2" t="n">
         <v>12.121121</v>
@@ -674,16 +683,16 @@
       <c r="M2"/>
       <c r="N2"/>
       <c r="O2" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P2" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q2"/>
       <c r="R2"/>
       <c r="S2"/>
       <c r="T2" t="s">
-        <v>84</v>
+        <v>85</v>
       </c>
       <c r="U2"/>
       <c r="V2"/>
@@ -720,10 +729,10 @@
       <c r="BA2"/>
       <c r="BB2"/>
       <c r="BC2" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BD2" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BE2"/>
       <c r="BF2"/>
@@ -736,24 +745,24 @@
       <c r="BM2"/>
       <c r="BN2"/>
       <c r="BO2" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BP2" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BQ2"/>
       <c r="BR2"/>
       <c r="BS2" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BT2" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BU2" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BV2" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BW2" t="n">
         <v>2015.0</v>
@@ -765,30 +774,33 @@
         <v>20.0</v>
       </c>
       <c r="BZ2" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="CA2" t="s">
-        <v>113</v>
+        <v>114</v>
+      </c>
+      <c r="CB2" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="3">
       <c r="A3" t="s">
-        <v>79</v>
+        <v>80</v>
       </c>
       <c r="B3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="C3" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D3" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E3" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F3" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G3" t="n">
         <v>12.123334</v>
@@ -807,16 +819,16 @@
       <c r="M3"/>
       <c r="N3"/>
       <c r="O3" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P3" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q3"/>
       <c r="R3"/>
       <c r="S3"/>
       <c r="T3" t="s">
-        <v>85</v>
+        <v>86</v>
       </c>
       <c r="U3"/>
       <c r="V3"/>
@@ -853,10 +865,10 @@
       <c r="BA3"/>
       <c r="BB3"/>
       <c r="BC3" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BD3" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BE3"/>
       <c r="BF3"/>
@@ -869,24 +881,24 @@
       <c r="BM3"/>
       <c r="BN3"/>
       <c r="BO3" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BP3" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BQ3"/>
       <c r="BR3"/>
       <c r="BS3" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BT3" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BU3" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BV3" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BW3" t="n">
         <v>2015.0</v>
@@ -898,30 +910,33 @@
         <v>21.0</v>
       </c>
       <c r="BZ3" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="CA3" t="s">
-        <v>113</v>
+        <v>114</v>
+      </c>
+      <c r="CB3" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="4">
       <c r="A4" t="s">
-        <v>80</v>
+        <v>81</v>
       </c>
       <c r="B4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="C4" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D4" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E4" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F4" t="s">
-        <v>98</v>
+        <v>99</v>
       </c>
       <c r="G4" t="n">
         <v>12.121121</v>
@@ -940,18 +955,18 @@
       <c r="M4"/>
       <c r="N4"/>
       <c r="O4" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P4" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q4"/>
       <c r="R4" t="s">
-        <v>102</v>
+        <v>103</v>
       </c>
       <c r="S4"/>
       <c r="T4" t="s">
-        <v>86</v>
+        <v>87</v>
       </c>
       <c r="U4"/>
       <c r="V4"/>
@@ -988,10 +1003,10 @@
       <c r="BA4"/>
       <c r="BB4"/>
       <c r="BC4" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BD4" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BE4"/>
       <c r="BF4"/>
@@ -1004,24 +1019,24 @@
       <c r="BM4"/>
       <c r="BN4"/>
       <c r="BO4" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BP4" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BQ4"/>
       <c r="BR4"/>
       <c r="BS4" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BT4" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BU4" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BV4" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BW4" t="n">
         <v>2015.0</v>
@@ -1033,30 +1048,33 @@
         <v>23.0</v>
       </c>
       <c r="BZ4" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="CA4" t="s">
-        <v>113</v>
+        <v>114</v>
+      </c>
+      <c r="CB4" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="5">
       <c r="A5" t="s">
-        <v>81</v>
+        <v>82</v>
       </c>
       <c r="B5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="C5" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D5" t="s">
-        <v>91</v>
+        <v>92</v>
       </c>
       <c r="E5" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F5" t="s">
-        <v>96</v>
+        <v>97</v>
       </c>
       <c r="G5" t="n">
         <v>12.121121</v>
@@ -1075,16 +1093,16 @@
       <c r="M5"/>
       <c r="N5"/>
       <c r="O5" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P5" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q5"/>
       <c r="R5"/>
       <c r="S5"/>
       <c r="T5" t="s">
-        <v>87</v>
+        <v>88</v>
       </c>
       <c r="U5"/>
       <c r="V5"/>
@@ -1121,10 +1139,10 @@
       <c r="BA5"/>
       <c r="BB5"/>
       <c r="BC5" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BD5" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BE5"/>
       <c r="BF5"/>
@@ -1137,24 +1155,24 @@
       <c r="BM5"/>
       <c r="BN5"/>
       <c r="BO5" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BP5" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BQ5"/>
       <c r="BR5"/>
       <c r="BS5" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BT5" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BU5" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BV5" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BW5" t="n">
         <v>2015.0</v>
@@ -1166,30 +1184,33 @@
         <v>20.0</v>
       </c>
       <c r="BZ5" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="CA5" t="s">
-        <v>113</v>
+        <v>114</v>
+      </c>
+      <c r="CB5" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="6">
       <c r="A6" t="s">
-        <v>82</v>
+        <v>83</v>
       </c>
       <c r="B6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="C6" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D6" t="s">
-        <v>92</v>
+        <v>93</v>
       </c>
       <c r="E6" t="s">
-        <v>95</v>
+        <v>96</v>
       </c>
       <c r="F6" t="s">
-        <v>97</v>
+        <v>98</v>
       </c>
       <c r="G6" t="n">
         <v>12.123334</v>
@@ -1208,16 +1229,16 @@
       <c r="M6"/>
       <c r="N6"/>
       <c r="O6" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P6" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q6"/>
       <c r="R6"/>
       <c r="S6"/>
       <c r="T6" t="s">
-        <v>88</v>
+        <v>89</v>
       </c>
       <c r="U6"/>
       <c r="V6"/>
@@ -1254,10 +1275,10 @@
       <c r="BA6"/>
       <c r="BB6"/>
       <c r="BC6" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BD6" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BE6"/>
       <c r="BF6"/>
@@ -1270,24 +1291,24 @@
       <c r="BM6"/>
       <c r="BN6"/>
       <c r="BO6" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BP6" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BQ6"/>
       <c r="BR6"/>
       <c r="BS6" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BT6" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BU6" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BV6" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BW6" t="n">
         <v>2015.0</v>
@@ -1299,30 +1320,33 @@
         <v>21.0</v>
       </c>
       <c r="BZ6" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="CA6" t="s">
-        <v>113</v>
+        <v>114</v>
+      </c>
+      <c r="CB6" t="s">
+        <v>115</v>
       </c>
     </row>
     <row r="7">
       <c r="A7" t="s">
-        <v>83</v>
+        <v>84</v>
       </c>
       <c r="B7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="C7" t="s">
-        <v>90</v>
+        <v>91</v>
       </c>
       <c r="D7" t="s">
-        <v>93</v>
+        <v>94</v>
       </c>
       <c r="E7" t="s">
-        <v>94</v>
+        <v>95</v>
       </c>
       <c r="F7" t="s">
-        <v>99</v>
+        <v>100</v>
       </c>
       <c r="G7" t="n">
         <v>12.121121</v>
@@ -1341,18 +1365,18 @@
       <c r="M7"/>
       <c r="N7"/>
       <c r="O7" t="s">
-        <v>100</v>
+        <v>101</v>
       </c>
       <c r="P7" t="s">
-        <v>101</v>
+        <v>102</v>
       </c>
       <c r="Q7"/>
       <c r="R7" t="s">
-        <v>103</v>
+        <v>104</v>
       </c>
       <c r="S7"/>
       <c r="T7" t="s">
-        <v>89</v>
+        <v>90</v>
       </c>
       <c r="U7"/>
       <c r="V7"/>
@@ -1389,10 +1413,10 @@
       <c r="BA7"/>
       <c r="BB7"/>
       <c r="BC7" t="s">
-        <v>104</v>
+        <v>105</v>
       </c>
       <c r="BD7" t="s">
-        <v>105</v>
+        <v>106</v>
       </c>
       <c r="BE7"/>
       <c r="BF7"/>
@@ -1405,24 +1429,24 @@
       <c r="BM7"/>
       <c r="BN7"/>
       <c r="BO7" t="s">
-        <v>106</v>
+        <v>107</v>
       </c>
       <c r="BP7" t="s">
-        <v>107</v>
+        <v>108</v>
       </c>
       <c r="BQ7"/>
       <c r="BR7"/>
       <c r="BS7" t="s">
-        <v>108</v>
+        <v>109</v>
       </c>
       <c r="BT7" t="s">
-        <v>109</v>
+        <v>110</v>
       </c>
       <c r="BU7" t="s">
-        <v>110</v>
+        <v>111</v>
       </c>
       <c r="BV7" t="s">
-        <v>111</v>
+        <v>112</v>
       </c>
       <c r="BW7" t="n">
         <v>2015.0</v>
@@ -1434,10 +1458,13 @@
         <v>23.0</v>
       </c>
       <c r="BZ7" t="s">
-        <v>112</v>
+        <v>113</v>
       </c>
       <c r="CA7" t="s">
-        <v>113</v>
+        <v>114</v>
+      </c>
+      <c r="CB7" t="s">
+        <v>115</v>
       </c>
     </row>
   </sheetData>

</xml_diff>